<commit_message>
Updated readme, .gitignore and file structure
Updated and moved readme files.
Updated .gitignore to omit 'temp_data' and 'output_data'
</commit_message>
<xml_diff>
--- a/main/test_data/p_clocked_times.xlsx
+++ b/main/test_data/p_clocked_times.xlsx
@@ -8,8 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Anders Bertilsson" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="3456" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Anders_Bertilsson" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Bertil Fredrik 9999" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>

</xml_diff>